<commit_message>
Saco la GOOGLE_API_KEY a un fichero
</commit_message>
<xml_diff>
--- a/.mio/ListadoRCs.xlsx
+++ b/.mio/ListadoRCs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
-  <workbookPr defaultThemeVersion="202300"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://totemtowers-my.sharepoint.com/personal/jose_lopezt_totemtowers_es/Documents/Documentos/desarrollo/python/EnrichAuction/.mio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\desarrollo\python\Subastas\enriqueceSubastas\.mio\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{292CCD0D-0861-4E05-869C-D5C771EA2C57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{084071F5-31AE-44DD-A4EC-AEF10483EE39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1164" yWindow="2040" windowWidth="17280" windowHeight="9960" xr2:uid="{811776C8-EF59-4F60-9CF4-DA4A35DAD93A}"/>
+    <workbookView xWindow="29010" yWindow="960" windowWidth="23175" windowHeight="11505" xr2:uid="{811776C8-EF59-4F60-9CF4-DA4A35DAD93A}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="54" uniqueCount="54">
   <si>
     <t>RC</t>
   </si>
@@ -195,6 +195,9 @@
   </si>
   <si>
     <t>19368A001002000000PM</t>
+  </si>
+  <si>
+    <t>7915008VK2881S0002GM</t>
   </si>
 </sst>
 </file>
@@ -566,273 +569,276 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{718FF057-7244-4378-B43E-AE7BF90CFFAF}">
-  <dimension ref="A1:A53"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D53"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.44140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+      <c r="D2" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
         <v>24</v>
       </c>
     </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="28" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="29" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="34" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A35" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
         <v>35</v>
       </c>
     </row>
-    <row r="37" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
         <v>36</v>
       </c>
     </row>
-    <row r="38" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="39" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="40" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
         <v>39</v>
       </c>
     </row>
-    <row r="41" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A41" t="s">
         <v>40</v>
       </c>
     </row>
-    <row r="42" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A42" t="s">
         <v>41</v>
       </c>
     </row>
-    <row r="43" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A43" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="44" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A44" t="s">
         <v>43</v>
       </c>
     </row>
-    <row r="45" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A45" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="46" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A46" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="47" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A47" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="48" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A48" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="49" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="50" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A50" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="51" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A51" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="52" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A52" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="53" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A53" t="s">
         <v>52</v>
       </c>

</xml_diff>